<commit_message>
add vul report data and modify file such as main.tex for v4
</commit_message>
<xml_diff>
--- a/ChatAFL-master/key_experiment/vulnerability/forked-daapd_漏洞发现_20260607124945.xlsx
+++ b/ChatAFL-master/key_experiment/vulnerability/forked-daapd_漏洞发现_20260607124945.xlsx
@@ -103,7 +103,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -126,6 +126,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -493,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J200"/>
+  <dimension ref="A1:K200"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -506,6 +509,7 @@
     <col width="70" customWidth="1" min="8" max="8"/>
     <col width="22" customWidth="1" min="9" max="9"/>
     <col width="65" customWidth="1" min="10" max="10"/>
+    <col width="65" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -557,6 +561,11 @@
       <c r="J1" s="1" t="inlineStr">
         <is>
           <t>为什么算漏洞</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>漏洞带来的影响</t>
         </is>
       </c>
     </row>
@@ -743,6 +752,13 @@
 5. 同版本已知CVE-2025-44560(9.8)和CVE-2021-38383(9.8)佐证内存安全问题</t>
         </is>
       </c>
+      <c r="K2" s="10" t="inlineStr">
+        <is>
+          <t>【远程代码执行风险】攻击者可构造恶意输入触发forked-daapd/owntone-server堆缓冲区溢出，覆盖相邻堆块的元数据或函数指针，进而劫持程序控制流，实现远程代码执行(RCE)。在ASAN编译环境下表现为SIGABRT崩溃，生产环境中可能导致任意代码执行。
+【拒绝服务(DoS)】即使攻击者未能成功利用RCE，每次恶意输入均会导致forked-daapd/owntone-server进程崩溃退出，造成服务不可用。若forked-daapd/owntone-server未配置自动重启或watchdog，服务将永久中断。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -893,6 +909,13 @@
 5. 同版本已知CVE-2025-44560(9.8)和CVE-2021-38383(9.8)佐证内存安全问题</t>
         </is>
       </c>
+      <c r="K3" s="10" t="inlineStr">
+        <is>
+          <t>【远程代码执行风险】攻击者可构造恶意输入触发forked-daapd/owntone-server堆缓冲区溢出，覆盖相邻堆块的元数据或函数指针，进而劫持程序控制流，实现远程代码执行(RCE)。在ASAN编译环境下表现为SIGABRT崩溃，生产环境中可能导致任意代码执行。
+【拒绝服务(DoS)】即使攻击者未能成功利用RCE，每次恶意输入均会导致forked-daapd/owntone-server进程崩溃退出，造成服务不可用。若forked-daapd/owntone-server未配置自动重启或watchdog，服务将永久中断。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1003,6 +1026,13 @@
 5. 同版本已知CVE-2025-44560(9.8)和CVE-2021-38383(9.8)佐证内存安全问题</t>
         </is>
       </c>
+      <c r="K4" s="10" t="inlineStr">
+        <is>
+          <t>【远程代码执行风险】攻击者可构造恶意输入触发forked-daapd/owntone-server堆缓冲区溢出，覆盖相邻堆块的元数据或函数指针，进而劫持程序控制流，实现远程代码执行(RCE)。在ASAN编译环境下表现为SIGABRT崩溃，生产环境中可能导致任意代码执行。
+【拒绝服务(DoS)】即使攻击者未能成功利用RCE，每次恶意输入均会导致forked-daapd/owntone-server进程崩溃退出，造成服务不可用。若forked-daapd/owntone-server未配置自动重启或watchdog，服务将永久中断。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1113,6 +1143,13 @@
 3. 10组独立实验每组均发现1-8个不同crash路径,跨组重叠率极低
 4. 种子包含畸形HTTP(二进制垃圾字节、CRLF注入、超大CL值等)
 5. 同版本已知CVE-2025-44560(9.8)和CVE-2021-38383(9.8)佐证内存安全问题</t>
+        </is>
+      </c>
+      <c r="K5" s="10" t="inlineStr">
+        <is>
+          <t>【远程代码执行风险】攻击者可构造恶意输入触发forked-daapd/owntone-server堆缓冲区溢出，覆盖相邻堆块的元数据或函数指针，进而劫持程序控制流，实现远程代码执行(RCE)。在ASAN编译环境下表现为SIGABRT崩溃，生产环境中可能导致任意代码执行。
+【拒绝服务(DoS)】即使攻击者未能成功利用RCE，每次恶意输入均会导致forked-daapd/owntone-server进程崩溃退出，造成服务不可用。若forked-daapd/owntone-server未配置自动重启或watchdog，服务将永久中断。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
         </is>
       </c>
     </row>
@@ -1252,6 +1289,13 @@
 5. 同版本已知CVE-2025-44560(9.8)和CVE-2021-38383(9.8)佐证内存安全问题</t>
         </is>
       </c>
+      <c r="K6" s="10" t="inlineStr">
+        <is>
+          <t>【远程代码执行风险】攻击者可构造恶意输入触发forked-daapd/owntone-server堆缓冲区溢出，覆盖相邻堆块的元数据或函数指针，进而劫持程序控制流，实现远程代码执行(RCE)。在ASAN编译环境下表现为SIGABRT崩溃，生产环境中可能导致任意代码执行。
+【拒绝服务(DoS)】即使攻击者未能成功利用RCE，每次恶意输入均会导致forked-daapd/owntone-server进程崩溃退出，造成服务不可用。若forked-daapd/owntone-server未配置自动重启或watchdog，服务将永久中断。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1373,6 +1417,13 @@
 5. 同版本已知CVE-2025-44560(9.8)和CVE-2021-38383(9.8)佐证内存安全问题</t>
         </is>
       </c>
+      <c r="K7" s="10" t="inlineStr">
+        <is>
+          <t>【远程代码执行风险】攻击者可构造恶意输入触发forked-daapd/owntone-server堆缓冲区溢出，覆盖相邻堆块的元数据或函数指针，进而劫持程序控制流，实现远程代码执行(RCE)。在ASAN编译环境下表现为SIGABRT崩溃，生产环境中可能导致任意代码执行。
+【拒绝服务(DoS)】即使攻击者未能成功利用RCE，每次恶意输入均会导致forked-daapd/owntone-server进程崩溃退出，造成服务不可用。若forked-daapd/owntone-server未配置自动重启或watchdog，服务将永久中断。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1497,6 +1548,13 @@
 5. 同版本已知CVE-2025-44560(9.8)和CVE-2021-38383(9.8)佐证内存安全问题</t>
         </is>
       </c>
+      <c r="K8" s="10" t="inlineStr">
+        <is>
+          <t>【远程代码执行风险】攻击者可构造恶意输入触发forked-daapd/owntone-server堆缓冲区溢出，覆盖相邻堆块的元数据或函数指针，进而劫持程序控制流，实现远程代码执行(RCE)。在ASAN编译环境下表现为SIGABRT崩溃，生产环境中可能导致任意代码执行。
+【拒绝服务(DoS)】即使攻击者未能成功利用RCE，每次恶意输入均会导致forked-daapd/owntone-server进程崩溃退出，造成服务不可用。若forked-daapd/owntone-server未配置自动重启或watchdog，服务将永久中断。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1599,6 +1657,13 @@
 3. 10组独立实验每组均发现1-8个不同crash路径,跨组重叠率极低
 4. 种子包含畸形HTTP(二进制垃圾字节、CRLF注入、超大CL值等)
 5. 同版本已知CVE-2025-44560(9.8)和CVE-2021-38383(9.8)佐证内存安全问题</t>
+        </is>
+      </c>
+      <c r="K9" s="10" t="inlineStr">
+        <is>
+          <t>【远程代码执行风险】攻击者可构造恶意输入触发forked-daapd/owntone-server堆缓冲区溢出，覆盖相邻堆块的元数据或函数指针，进而劫持程序控制流，实现远程代码执行(RCE)。在ASAN编译环境下表现为SIGABRT崩溃，生产环境中可能导致任意代码执行。
+【拒绝服务(DoS)】即使攻击者未能成功利用RCE，每次恶意输入均会导致forked-daapd/owntone-server进程崩溃退出，造成服务不可用。若forked-daapd/owntone-server未配置自动重启或watchdog，服务将永久中断。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
         </is>
       </c>
     </row>
@@ -1729,6 +1794,13 @@
 5. 同版本已知CVE-2025-44560(9.8)和CVE-2021-38383(9.8)佐证内存安全问题</t>
         </is>
       </c>
+      <c r="K10" s="10" t="inlineStr">
+        <is>
+          <t>【远程代码执行风险】攻击者可构造恶意输入触发forked-daapd/owntone-server堆缓冲区溢出，覆盖相邻堆块的元数据或函数指针，进而劫持程序控制流，实现远程代码执行(RCE)。在ASAN编译环境下表现为SIGABRT崩溃，生产环境中可能导致任意代码执行。
+【拒绝服务(DoS)】即使攻击者未能成功利用RCE，每次恶意输入均会导致forked-daapd/owntone-server进程崩溃退出，造成服务不可用。若forked-daapd/owntone-server未配置自动重启或watchdog，服务将永久中断。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1841,6 +1913,13 @@
 5. 同版本已知CVE-2025-44560(9.8)和CVE-2021-38383(9.8)佐证内存安全问题</t>
         </is>
       </c>
+      <c r="K11" s="10" t="inlineStr">
+        <is>
+          <t>【远程代码执行风险】攻击者可构造恶意输入触发forked-daapd/owntone-server堆缓冲区溢出，覆盖相邻堆块的元数据或函数指针，进而劫持程序控制流，实现远程代码执行(RCE)。在ASAN编译环境下表现为SIGABRT崩溃，生产环境中可能导致任意代码执行。
+【拒绝服务(DoS)】即使攻击者未能成功利用RCE，每次恶意输入均会导致forked-daapd/owntone-server进程崩溃退出，造成服务不可用。若forked-daapd/owntone-server未配置自动重启或watchdog，服务将永久中断。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1947,6 +2026,13 @@
 5. 同版本已知CVE-2025-44560(9.8)和CVE-2021-38383(9.8)佐证内存安全问题</t>
         </is>
       </c>
+      <c r="K12" s="10" t="inlineStr">
+        <is>
+          <t>【远程代码执行风险】攻击者可构造恶意输入触发forked-daapd/owntone-server堆缓冲区溢出，覆盖相邻堆块的元数据或函数指针，进而劫持程序控制流，实现远程代码执行(RCE)。在ASAN编译环境下表现为SIGABRT崩溃，生产环境中可能导致任意代码执行。
+【拒绝服务(DoS)】即使攻击者未能成功利用RCE，每次恶意输入均会导致forked-daapd/owntone-server进程崩溃退出，造成服务不可用。若forked-daapd/owntone-server未配置自动重启或watchdog，服务将永久中断。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -2065,6 +2151,13 @@
 5. 同版本已知CVE-2025-44560(9.8)和CVE-2021-38383(9.8)佐证内存安全问题</t>
         </is>
       </c>
+      <c r="K13" s="10" t="inlineStr">
+        <is>
+          <t>【远程代码执行风险】攻击者可构造恶意输入触发forked-daapd/owntone-server堆缓冲区溢出，覆盖相邻堆块的元数据或函数指针，进而劫持程序控制流，实现远程代码执行(RCE)。在ASAN编译环境下表现为SIGABRT崩溃，生产环境中可能导致任意代码执行。
+【拒绝服务(DoS)】即使攻击者未能成功利用RCE，每次恶意输入均会导致forked-daapd/owntone-server进程崩溃退出，造成服务不可用。若forked-daapd/owntone-server未配置自动重启或watchdog，服务将永久中断。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -2191,6 +2284,13 @@
 5. 同版本已知CVE-2025-44560(9.8)和CVE-2021-38383(9.8)佐证内存安全问题</t>
         </is>
       </c>
+      <c r="K14" s="10" t="inlineStr">
+        <is>
+          <t>【远程代码执行风险】攻击者可构造恶意输入触发forked-daapd/owntone-server堆缓冲区溢出，覆盖相邻堆块的元数据或函数指针，进而劫持程序控制流，实现远程代码执行(RCE)。在ASAN编译环境下表现为SIGABRT崩溃，生产环境中可能导致任意代码执行。
+【拒绝服务(DoS)】即使攻击者未能成功利用RCE，每次恶意输入均会导致forked-daapd/owntone-server进程崩溃退出，造成服务不可用。若forked-daapd/owntone-server未配置自动重启或watchdog，服务将永久中断。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -2290,6 +2390,13 @@
 5. 同版本已知CVE-2025-44560(9.8)和CVE-2021-38383(9.8)佐证内存安全问题</t>
         </is>
       </c>
+      <c r="K15" s="10" t="inlineStr">
+        <is>
+          <t>【远程代码执行风险】攻击者可构造恶意输入触发forked-daapd/owntone-server堆缓冲区溢出，覆盖相邻堆块的元数据或函数指针，进而劫持程序控制流，实现远程代码执行(RCE)。在ASAN编译环境下表现为SIGABRT崩溃，生产环境中可能导致任意代码执行。
+【拒绝服务(DoS)】即使攻击者未能成功利用RCE，每次恶意输入均会导致forked-daapd/owntone-server进程崩溃退出，造成服务不可用。若forked-daapd/owntone-server未配置自动重启或watchdog，服务将永久中断。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -2411,6 +2518,13 @@
 5. 同版本已知CVE-2025-44560(9.8)和CVE-2021-38383(9.8)佐证内存安全问题</t>
         </is>
       </c>
+      <c r="K16" s="10" t="inlineStr">
+        <is>
+          <t>【远程代码执行风险】攻击者可构造恶意输入触发forked-daapd/owntone-server堆缓冲区溢出，覆盖相邻堆块的元数据或函数指针，进而劫持程序控制流，实现远程代码执行(RCE)。在ASAN编译环境下表现为SIGABRT崩溃，生产环境中可能导致任意代码执行。
+【拒绝服务(DoS)】即使攻击者未能成功利用RCE，每次恶意输入均会导致forked-daapd/owntone-server进程崩溃退出，造成服务不可用。若forked-daapd/owntone-server未配置自动重启或watchdog，服务将永久中断。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -2533,6 +2647,13 @@
 5. 同版本已知CVE-2025-44560(9.8)和CVE-2021-38383(9.8)佐证内存安全问题</t>
         </is>
       </c>
+      <c r="K17" s="10" t="inlineStr">
+        <is>
+          <t>【远程代码执行风险】攻击者可构造恶意输入触发forked-daapd/owntone-server堆缓冲区溢出，覆盖相邻堆块的元数据或函数指针，进而劫持程序控制流，实现远程代码执行(RCE)。在ASAN编译环境下表现为SIGABRT崩溃，生产环境中可能导致任意代码执行。
+【拒绝服务(DoS)】即使攻击者未能成功利用RCE，每次恶意输入均会导致forked-daapd/owntone-server进程崩溃退出，造成服务不可用。若forked-daapd/owntone-server未配置自动重启或watchdog，服务将永久中断。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -2700,6 +2821,13 @@
 3. 10组独立实验每组均发现1-8个不同crash路径,跨组重叠率极低
 4. 种子包含畸形HTTP(二进制垃圾字节、CRLF注入、超大CL值等)
 5. 同版本已知CVE-2025-44560(9.8)和CVE-2021-38383(9.8)佐证内存安全问题</t>
+        </is>
+      </c>
+      <c r="K18" s="10" t="inlineStr">
+        <is>
+          <t>【远程代码执行风险】攻击者可构造恶意输入触发forked-daapd/owntone-server堆缓冲区溢出，覆盖相邻堆块的元数据或函数指针，进而劫持程序控制流，实现远程代码执行(RCE)。在ASAN编译环境下表现为SIGABRT崩溃，生产环境中可能导致任意代码执行。
+【拒绝服务(DoS)】即使攻击者未能成功利用RCE，每次恶意输入均会导致forked-daapd/owntone-server进程崩溃退出，造成服务不可用。若forked-daapd/owntone-server未配置自动重启或watchdog，服务将永久中断。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
         </is>
       </c>
     </row>
@@ -2837,6 +2965,13 @@
 5. 同版本已知CVE-2025-44560(9.8)和CVE-2021-38383(9.8)佐证内存安全问题</t>
         </is>
       </c>
+      <c r="K19" s="10" t="inlineStr">
+        <is>
+          <t>【远程代码执行风险】攻击者可构造恶意输入触发forked-daapd/owntone-server堆缓冲区溢出，覆盖相邻堆块的元数据或函数指针，进而劫持程序控制流，实现远程代码执行(RCE)。在ASAN编译环境下表现为SIGABRT崩溃，生产环境中可能导致任意代码执行。
+【拒绝服务(DoS)】即使攻击者未能成功利用RCE，每次恶意输入均会导致forked-daapd/owntone-server进程崩溃退出，造成服务不可用。若forked-daapd/owntone-server未配置自动重启或watchdog，服务将永久中断。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -2965,6 +3100,13 @@
 5. 同版本已知CVE-2025-44560(9.8)和CVE-2021-38383(9.8)佐证内存安全问题</t>
         </is>
       </c>
+      <c r="K20" s="10" t="inlineStr">
+        <is>
+          <t>【远程代码执行风险】攻击者可构造恶意输入触发forked-daapd/owntone-server堆缓冲区溢出，覆盖相邻堆块的元数据或函数指针，进而劫持程序控制流，实现远程代码执行(RCE)。在ASAN编译环境下表现为SIGABRT崩溃，生产环境中可能导致任意代码执行。
+【拒绝服务(DoS)】即使攻击者未能成功利用RCE，每次恶意输入均会导致forked-daapd/owntone-server进程崩溃退出，造成服务不可用。若forked-daapd/owntone-server未配置自动重启或watchdog，服务将永久中断。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -3071,6 +3213,13 @@
 5. 同版本已知CVE-2025-44560(9.8)和CVE-2021-38383(9.8)佐证内存安全问题</t>
         </is>
       </c>
+      <c r="K21" s="10" t="inlineStr">
+        <is>
+          <t>【远程代码执行风险】攻击者可构造恶意输入触发forked-daapd/owntone-server堆缓冲区溢出，覆盖相邻堆块的元数据或函数指针，进而劫持程序控制流，实现远程代码执行(RCE)。在ASAN编译环境下表现为SIGABRT崩溃，生产环境中可能导致任意代码执行。
+【拒绝服务(DoS)】即使攻击者未能成功利用RCE，每次恶意输入均会导致forked-daapd/owntone-server进程崩溃退出，造成服务不可用。若forked-daapd/owntone-server未配置自动重启或watchdog，服务将永久中断。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -3172,6 +3321,13 @@
 5. 同版本已知CVE-2025-44560(9.8)和CVE-2021-38383(9.8)佐证内存安全问题</t>
         </is>
       </c>
+      <c r="K22" s="10" t="inlineStr">
+        <is>
+          <t>【远程代码执行风险】攻击者可构造恶意输入触发forked-daapd/owntone-server堆缓冲区溢出，覆盖相邻堆块的元数据或函数指针，进而劫持程序控制流，实现远程代码执行(RCE)。在ASAN编译环境下表现为SIGABRT崩溃，生产环境中可能导致任意代码执行。
+【拒绝服务(DoS)】即使攻击者未能成功利用RCE，每次恶意输入均会导致forked-daapd/owntone-server进程崩溃退出，造成服务不可用。若forked-daapd/owntone-server未配置自动重启或watchdog，服务将永久中断。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -3271,6 +3427,13 @@
 5. 同版本已知CVE-2025-44560(9.8)和CVE-2021-38383(9.8)佐证内存安全问题</t>
         </is>
       </c>
+      <c r="K23" s="10" t="inlineStr">
+        <is>
+          <t>【远程代码执行风险】攻击者可构造恶意输入触发forked-daapd/owntone-server堆缓冲区溢出，覆盖相邻堆块的元数据或函数指针，进而劫持程序控制流，实现远程代码执行(RCE)。在ASAN编译环境下表现为SIGABRT崩溃，生产环境中可能导致任意代码执行。
+【拒绝服务(DoS)】即使攻击者未能成功利用RCE，每次恶意输入均会导致forked-daapd/owntone-server进程崩溃退出，造成服务不可用。若forked-daapd/owntone-server未配置自动重启或watchdog，服务将永久中断。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -3417,6 +3580,13 @@
 5. 同版本已知CVE-2025-44560(9.8)和CVE-2021-38383(9.8)佐证内存安全问题</t>
         </is>
       </c>
+      <c r="K24" s="10" t="inlineStr">
+        <is>
+          <t>【远程代码执行风险】攻击者可构造恶意输入触发forked-daapd/owntone-server堆缓冲区溢出，覆盖相邻堆块的元数据或函数指针，进而劫持程序控制流，实现远程代码执行(RCE)。在ASAN编译环境下表现为SIGABRT崩溃，生产环境中可能导致任意代码执行。
+【拒绝服务(DoS)】即使攻击者未能成功利用RCE，每次恶意输入均会导致forked-daapd/owntone-server进程崩溃退出，造成服务不可用。若forked-daapd/owntone-server未配置自动重启或watchdog，服务将永久中断。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -3530,6 +3700,13 @@
 5. 同版本已知CVE-2025-44560(9.8)和CVE-2021-38383(9.8)佐证内存安全问题</t>
         </is>
       </c>
+      <c r="K25" s="10" t="inlineStr">
+        <is>
+          <t>【远程代码执行风险】攻击者可构造恶意输入触发forked-daapd/owntone-server堆缓冲区溢出，覆盖相邻堆块的元数据或函数指针，进而劫持程序控制流，实现远程代码执行(RCE)。在ASAN编译环境下表现为SIGABRT崩溃，生产环境中可能导致任意代码执行。
+【拒绝服务(DoS)】即使攻击者未能成功利用RCE，每次恶意输入均会导致forked-daapd/owntone-server进程崩溃退出，造成服务不可用。若forked-daapd/owntone-server未配置自动重启或watchdog，服务将永久中断。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -3673,6 +3850,13 @@
 5. 同版本已知CVE-2025-44560(9.8)和CVE-2021-38383(9.8)佐证内存安全问题</t>
         </is>
       </c>
+      <c r="K26" s="10" t="inlineStr">
+        <is>
+          <t>【远程代码执行风险】攻击者可构造恶意输入触发forked-daapd/owntone-server堆缓冲区溢出，覆盖相邻堆块的元数据或函数指针，进而劫持程序控制流，实现远程代码执行(RCE)。在ASAN编译环境下表现为SIGABRT崩溃，生产环境中可能导致任意代码执行。
+【拒绝服务(DoS)】即使攻击者未能成功利用RCE，每次恶意输入均会导致forked-daapd/owntone-server进程崩溃退出，造成服务不可用。若forked-daapd/owntone-server未配置自动重启或watchdog，服务将永久中断。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -3835,6 +4019,13 @@
 5. 同版本已知CVE-2025-44560(9.8)和CVE-2021-38383(9.8)佐证内存安全问题</t>
         </is>
       </c>
+      <c r="K27" s="10" t="inlineStr">
+        <is>
+          <t>【远程代码执行风险】攻击者可构造恶意输入触发forked-daapd/owntone-server堆缓冲区溢出，覆盖相邻堆块的元数据或函数指针，进而劫持程序控制流，实现远程代码执行(RCE)。在ASAN编译环境下表现为SIGABRT崩溃，生产环境中可能导致任意代码执行。
+【拒绝服务(DoS)】即使攻击者未能成功利用RCE，每次恶意输入均会导致forked-daapd/owntone-server进程崩溃退出，造成服务不可用。若forked-daapd/owntone-server未配置自动重启或watchdog，服务将永久中断。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -3934,6 +4125,13 @@
 5. 同版本已知CVE-2025-44560(9.8)和CVE-2021-38383(9.8)佐证内存安全问题</t>
         </is>
       </c>
+      <c r="K28" s="10" t="inlineStr">
+        <is>
+          <t>【远程代码执行风险】攻击者可构造恶意输入触发forked-daapd/owntone-server堆缓冲区溢出，覆盖相邻堆块的元数据或函数指针，进而劫持程序控制流，实现远程代码执行(RCE)。在ASAN编译环境下表现为SIGABRT崩溃，生产环境中可能导致任意代码执行。
+【拒绝服务(DoS)】即使攻击者未能成功利用RCE，每次恶意输入均会导致forked-daapd/owntone-server进程崩溃退出，造成服务不可用。若forked-daapd/owntone-server未配置自动重启或watchdog，服务将永久中断。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -4034,6 +4232,13 @@
 5. 同版本已知CVE-2025-44560(9.8)和CVE-2021-38383(9.8)佐证内存安全问题</t>
         </is>
       </c>
+      <c r="K29" s="10" t="inlineStr">
+        <is>
+          <t>【远程代码执行风险】攻击者可构造恶意输入触发forked-daapd/owntone-server堆缓冲区溢出，覆盖相邻堆块的元数据或函数指针，进而劫持程序控制流，实现远程代码执行(RCE)。在ASAN编译环境下表现为SIGABRT崩溃，生产环境中可能导致任意代码执行。
+【拒绝服务(DoS)】即使攻击者未能成功利用RCE，每次恶意输入均会导致forked-daapd/owntone-server进程崩溃退出，造成服务不可用。若forked-daapd/owntone-server未配置自动重启或watchdog，服务将永久中断。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -4134,6 +4339,13 @@
 5. 同版本已知CVE-2025-44560(9.8)和CVE-2021-38383(9.8)佐证内存安全问题</t>
         </is>
       </c>
+      <c r="K30" s="10" t="inlineStr">
+        <is>
+          <t>【远程代码执行风险】攻击者可构造恶意输入触发forked-daapd/owntone-server堆缓冲区溢出，覆盖相邻堆块的元数据或函数指针，进而劫持程序控制流，实现远程代码执行(RCE)。在ASAN编译环境下表现为SIGABRT崩溃，生产环境中可能导致任意代码执行。
+【拒绝服务(DoS)】即使攻击者未能成功利用RCE，每次恶意输入均会导致forked-daapd/owntone-server进程崩溃退出，造成服务不可用。若forked-daapd/owntone-server未配置自动重启或watchdog，服务将永久中断。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -4233,6 +4445,13 @@
 5. 同版本已知CVE-2025-44560(9.8)和CVE-2021-38383(9.8)佐证内存安全问题</t>
         </is>
       </c>
+      <c r="K31" s="10" t="inlineStr">
+        <is>
+          <t>【远程代码执行风险】攻击者可构造恶意输入触发forked-daapd/owntone-server堆缓冲区溢出，覆盖相邻堆块的元数据或函数指针，进而劫持程序控制流，实现远程代码执行(RCE)。在ASAN编译环境下表现为SIGABRT崩溃，生产环境中可能导致任意代码执行。
+【拒绝服务(DoS)】即使攻击者未能成功利用RCE，每次恶意输入均会导致forked-daapd/owntone-server进程崩溃退出，造成服务不可用。若forked-daapd/owntone-server未配置自动重启或watchdog，服务将永久中断。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -4331,6 +4550,13 @@
 5. 同版本已知CVE-2025-44560(9.8)和CVE-2021-38383(9.8)佐证内存安全问题</t>
         </is>
       </c>
+      <c r="K32" s="10" t="inlineStr">
+        <is>
+          <t>【远程代码执行风险】攻击者可构造恶意输入触发forked-daapd/owntone-server堆缓冲区溢出，覆盖相邻堆块的元数据或函数指针，进而劫持程序控制流，实现远程代码执行(RCE)。在ASAN编译环境下表现为SIGABRT崩溃，生产环境中可能导致任意代码执行。
+【拒绝服务(DoS)】即使攻击者未能成功利用RCE，每次恶意输入均会导致forked-daapd/owntone-server进程崩溃退出，造成服务不可用。若forked-daapd/owntone-server未配置自动重启或watchdog，服务将永久中断。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -4428,6 +4654,13 @@
 5. 同版本已知CVE-2025-44560(9.8)和CVE-2021-38383(9.8)佐证内存安全问题</t>
         </is>
       </c>
+      <c r="K33" s="10" t="inlineStr">
+        <is>
+          <t>【远程代码执行风险】攻击者可构造恶意输入触发forked-daapd/owntone-server堆缓冲区溢出，覆盖相邻堆块的元数据或函数指针，进而劫持程序控制流，实现远程代码执行(RCE)。在ASAN编译环境下表现为SIGABRT崩溃，生产环境中可能导致任意代码执行。
+【拒绝服务(DoS)】即使攻击者未能成功利用RCE，每次恶意输入均会导致forked-daapd/owntone-server进程崩溃退出，造成服务不可用。若forked-daapd/owntone-server未配置自动重启或watchdog，服务将永久中断。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -4527,6 +4760,13 @@
 5. 同版本已知CVE-2025-44560(9.8)和CVE-2021-38383(9.8)佐证内存安全问题</t>
         </is>
       </c>
+      <c r="K34" s="10" t="inlineStr">
+        <is>
+          <t>【远程代码执行风险】攻击者可构造恶意输入触发forked-daapd/owntone-server堆缓冲区溢出，覆盖相邻堆块的元数据或函数指针，进而劫持程序控制流，实现远程代码执行(RCE)。在ASAN编译环境下表现为SIGABRT崩溃，生产环境中可能导致任意代码执行。
+【拒绝服务(DoS)】即使攻击者未能成功利用RCE，每次恶意输入均会导致forked-daapd/owntone-server进程崩溃退出，造成服务不可用。若forked-daapd/owntone-server未配置自动重启或watchdog，服务将永久中断。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -4629,6 +4869,13 @@
 5. 同版本已知CVE-2025-44560(9.8)和CVE-2021-38383(9.8)佐证内存安全问题</t>
         </is>
       </c>
+      <c r="K35" s="10" t="inlineStr">
+        <is>
+          <t>【远程代码执行风险】攻击者可构造恶意输入触发forked-daapd/owntone-server堆缓冲区溢出，覆盖相邻堆块的元数据或函数指针，进而劫持程序控制流，实现远程代码执行(RCE)。在ASAN编译环境下表现为SIGABRT崩溃，生产环境中可能导致任意代码执行。
+【拒绝服务(DoS)】即使攻击者未能成功利用RCE，每次恶意输入均会导致forked-daapd/owntone-server进程崩溃退出，造成服务不可用。若forked-daapd/owntone-server未配置自动重启或watchdog，服务将永久中断。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -4748,6 +4995,13 @@
 5. 同版本已知CVE-2025-44560(9.8)和CVE-2021-38383(9.8)佐证内存安全问题</t>
         </is>
       </c>
+      <c r="K36" s="10" t="inlineStr">
+        <is>
+          <t>【远程代码执行风险】攻击者可构造恶意输入触发forked-daapd/owntone-server堆缓冲区溢出，覆盖相邻堆块的元数据或函数指针，进而劫持程序控制流，实现远程代码执行(RCE)。在ASAN编译环境下表现为SIGABRT崩溃，生产环境中可能导致任意代码执行。
+【拒绝服务(DoS)】即使攻击者未能成功利用RCE，每次恶意输入均会导致forked-daapd/owntone-server进程崩溃退出，造成服务不可用。若forked-daapd/owntone-server未配置自动重启或watchdog，服务将永久中断。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -4847,6 +5101,13 @@
 5. 同版本已知CVE-2025-44560(9.8)和CVE-2021-38383(9.8)佐证内存安全问题</t>
         </is>
       </c>
+      <c r="K37" s="10" t="inlineStr">
+        <is>
+          <t>【远程代码执行风险】攻击者可构造恶意输入触发forked-daapd/owntone-server堆缓冲区溢出，覆盖相邻堆块的元数据或函数指针，进而劫持程序控制流，实现远程代码执行(RCE)。在ASAN编译环境下表现为SIGABRT崩溃，生产环境中可能导致任意代码执行。
+【拒绝服务(DoS)】即使攻击者未能成功利用RCE，每次恶意输入均会导致forked-daapd/owntone-server进程崩溃退出，造成服务不可用。若forked-daapd/owntone-server未配置自动重启或watchdog，服务将永久中断。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -4953,6 +5214,13 @@
 5. 同版本已知CVE-2025-44560(9.8)和CVE-2021-38383(9.8)佐证内存安全问题</t>
         </is>
       </c>
+      <c r="K38" s="10" t="inlineStr">
+        <is>
+          <t>【远程代码执行风险】攻击者可构造恶意输入触发forked-daapd/owntone-server堆缓冲区溢出，覆盖相邻堆块的元数据或函数指针，进而劫持程序控制流，实现远程代码执行(RCE)。在ASAN编译环境下表现为SIGABRT崩溃，生产环境中可能导致任意代码执行。
+【拒绝服务(DoS)】即使攻击者未能成功利用RCE，每次恶意输入均会导致forked-daapd/owntone-server进程崩溃退出，造成服务不可用。若forked-daapd/owntone-server未配置自动重启或watchdog，服务将永久中断。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -5051,6 +5319,13 @@
 5. 同版本已知CVE-2025-44560(9.8)和CVE-2021-38383(9.8)佐证内存安全问题</t>
         </is>
       </c>
+      <c r="K39" s="10" t="inlineStr">
+        <is>
+          <t>【远程代码执行风险】攻击者可构造恶意输入触发forked-daapd/owntone-server堆缓冲区溢出，覆盖相邻堆块的元数据或函数指针，进而劫持程序控制流，实现远程代码执行(RCE)。在ASAN编译环境下表现为SIGABRT崩溃，生产环境中可能导致任意代码执行。
+【拒绝服务(DoS)】即使攻击者未能成功利用RCE，每次恶意输入均会导致forked-daapd/owntone-server进程崩溃退出，造成服务不可用。若forked-daapd/owntone-server未配置自动重启或watchdog，服务将永久中断。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -5173,6 +5448,13 @@
 5. 同版本已知CVE-2025-44560(9.8)和CVE-2021-38383(9.8)佐证内存安全问题</t>
         </is>
       </c>
+      <c r="K40" s="10" t="inlineStr">
+        <is>
+          <t>【远程代码执行风险】攻击者可构造恶意输入触发forked-daapd/owntone-server堆缓冲区溢出，覆盖相邻堆块的元数据或函数指针，进而劫持程序控制流，实现远程代码执行(RCE)。在ASAN编译环境下表现为SIGABRT崩溃，生产环境中可能导致任意代码执行。
+【拒绝服务(DoS)】即使攻击者未能成功利用RCE，每次恶意输入均会导致forked-daapd/owntone-server进程崩溃退出，造成服务不可用。若forked-daapd/owntone-server未配置自动重启或watchdog，服务将永久中断。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
@@ -5435,6 +5717,14 @@
 5. 独立复现确认: replay_logical_vuln.sh — 71+ oracle违规验证</t>
         </is>
       </c>
+      <c r="K41" s="10" t="inlineStr">
+        <is>
+          <t>【HTTP缓存投毒】攻击者可利用forked-daapd/owntone-server的HTTP请求走私/响应分割漏洞，向前端缓存/代理服务器注入恶意HTTP响应，污染缓存内容。后续合法用户请求将收到被篡改的缓存内容，可能导致XSS、恶意重定向或恶意文件下载。
+【会话劫持与凭证窃取】通过HTTP响应头注入，攻击者可构造恶意响应设置Cookie、重定向用户到钓鱼页面，或注入恶意JavaScript代码窃取用户会话令牌和登录凭证。
+【WAF/安全设备绕过】前端代理与后端forked-daapd/owntone-server对HTTP请求边界解析不一致，允许恶意请求绕过Web应用防火墙(WAF)的检测规则，直接到达后端服务器。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
@@ -5666,6 +5956,14 @@
 5. 独立复现确认: replay_logical_vuln.sh — 71+ oracle违规验证</t>
         </is>
       </c>
+      <c r="K42" s="10" t="inlineStr">
+        <is>
+          <t>【HTTP缓存投毒】攻击者可利用forked-daapd/owntone-server的HTTP请求走私/响应分割漏洞，向前端缓存/代理服务器注入恶意HTTP响应，污染缓存内容。后续合法用户请求将收到被篡改的缓存内容，可能导致XSS、恶意重定向或恶意文件下载。
+【会话劫持与凭证窃取】通过HTTP响应头注入，攻击者可构造恶意响应设置Cookie、重定向用户到钓鱼页面，或注入恶意JavaScript代码窃取用户会话令牌和登录凭证。
+【WAF/安全设备绕过】前端代理与后端forked-daapd/owntone-server对HTTP请求边界解析不一致，允许恶意请求绕过Web应用防火墙(WAF)的检测规则，直接到达后端服务器。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
@@ -5848,6 +6146,14 @@
 5. 独立复现确认: replay_logical_vuln.sh — 8+ oracle违规验证</t>
         </is>
       </c>
+      <c r="K43" s="10" t="inlineStr">
+        <is>
+          <t>【HTTP缓存投毒】攻击者可利用forked-daapd/owntone-server的HTTP请求走私/响应分割漏洞，向前端缓存/代理服务器注入恶意HTTP响应，污染缓存内容。后续合法用户请求将收到被篡改的缓存内容，可能导致XSS、恶意重定向或恶意文件下载。
+【会话劫持与凭证窃取】通过HTTP响应头注入，攻击者可构造恶意响应设置Cookie、重定向用户到钓鱼页面，或注入恶意JavaScript代码窃取用户会话令牌和登录凭证。
+【WAF/安全设备绕过】前端代理与后端forked-daapd/owntone-server对HTTP请求边界解析不一致，允许恶意请求绕过Web应用防火墙(WAF)的检测规则，直接到达后端服务器。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
@@ -5976,6 +6282,14 @@
 3. 攻击者可利用此绕过WAF/安全控制,窃取其他用户数据
 4. AFLNet协议Oracle在fuzzing中检测到CL desync违规
 5. 独立复现确认: replay_logical_vuln.sh — 71+ oracle违规验证</t>
+        </is>
+      </c>
+      <c r="K44" s="10" t="inlineStr">
+        <is>
+          <t>【HTTP缓存投毒】攻击者可利用forked-daapd/owntone-server的HTTP请求走私/响应分割漏洞，向前端缓存/代理服务器注入恶意HTTP响应，污染缓存内容。后续合法用户请求将收到被篡改的缓存内容，可能导致XSS、恶意重定向或恶意文件下载。
+【会话劫持与凭证窃取】通过HTTP响应头注入，攻击者可构造恶意响应设置Cookie、重定向用户到钓鱼页面，或注入恶意JavaScript代码窃取用户会话令牌和登录凭证。
+【WAF/安全设备绕过】前端代理与后端forked-daapd/owntone-server对HTTP请求边界解析不一致，允许恶意请求绕过Web应用防火墙(WAF)的检测规则，直接到达后端服务器。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
         </is>
       </c>
     </row>
@@ -6130,6 +6444,14 @@
 5. 独立复现确认: replay_logical_vuln.sh — 8+ oracle违规验证</t>
         </is>
       </c>
+      <c r="K45" s="10" t="inlineStr">
+        <is>
+          <t>【HTTP缓存投毒】攻击者可利用forked-daapd/owntone-server的HTTP请求走私/响应分割漏洞，向前端缓存/代理服务器注入恶意HTTP响应，污染缓存内容。后续合法用户请求将收到被篡改的缓存内容，可能导致XSS、恶意重定向或恶意文件下载。
+【会话劫持与凭证窃取】通过HTTP响应头注入，攻击者可构造恶意响应设置Cookie、重定向用户到钓鱼页面，或注入恶意JavaScript代码窃取用户会话令牌和登录凭证。
+【WAF/安全设备绕过】前端代理与后端forked-daapd/owntone-server对HTTP请求边界解析不一致，允许恶意请求绕过Web应用防火墙(WAF)的检测规则，直接到达后端服务器。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
@@ -6344,6 +6666,14 @@
 5. 独立复现确认: replay_logical_vuln.sh — 200 OK响应确认绕过</t>
         </is>
       </c>
+      <c r="K46" s="10" t="inlineStr">
+        <is>
+          <t>【未授权访问】攻击者可绕过forked-daapd/owntone-server的身份认证机制，无需提供有效凭据即可访问受保护的服务功能和数据。这相当于将forked-daapd/owntone-server的认证门控完全失效，任何能够网络连接到服务的攻击者均可获得已认证用户的权限。
+【数据泄露与篡改】认证绕过后，攻击者可读取、修改、删除forked-daapd/owntone-server管理的所有数据，包括敏感配置文件、用户数据、媒体内容等。若forked-daapd/owntone-server连接到其他后端系统，攻击面将进一步扩大。
+【权限提升跳板】认证绕过通常可作为进一步攻击的跳板——攻击者获取立足点后可利用其他漏洞（如路径遍历、命令注入）扩大控制范围。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
@@ -6606,6 +6936,14 @@
 3. 攻击者可利用此绕过WAF/安全控制,窃取其他用户数据
 4. AFLNet协议Oracle在fuzzing中检测到CL desync违规
 5. 独立复现确认: replay_logical_vuln.sh — 71+ oracle违规验证</t>
+        </is>
+      </c>
+      <c r="K47" s="10" t="inlineStr">
+        <is>
+          <t>【HTTP缓存投毒】攻击者可利用forked-daapd/owntone-server的HTTP请求走私/响应分割漏洞，向前端缓存/代理服务器注入恶意HTTP响应，污染缓存内容。后续合法用户请求将收到被篡改的缓存内容，可能导致XSS、恶意重定向或恶意文件下载。
+【会话劫持与凭证窃取】通过HTTP响应头注入，攻击者可构造恶意响应设置Cookie、重定向用户到钓鱼页面，或注入恶意JavaScript代码窃取用户会话令牌和登录凭证。
+【WAF/安全设备绕过】前端代理与后端forked-daapd/owntone-server对HTTP请求边界解析不一致，允许恶意请求绕过Web应用防火墙(WAF)的检测规则，直接到达后端服务器。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
         </is>
       </c>
     </row>
@@ -6813,6 +7151,14 @@
 3. HTTP响应分割可导致缓存投毒、跨站脚本、页面劫持
 4. AFLNet协议Oracle检测到嵌入式HTTP响应模式
 5. 独立复现确认: replay_logical_vuln.sh — 8+ oracle违规验证</t>
+        </is>
+      </c>
+      <c r="K48" s="10" t="inlineStr">
+        <is>
+          <t>【HTTP缓存投毒】攻击者可利用forked-daapd/owntone-server的HTTP请求走私/响应分割漏洞，向前端缓存/代理服务器注入恶意HTTP响应，污染缓存内容。后续合法用户请求将收到被篡改的缓存内容，可能导致XSS、恶意重定向或恶意文件下载。
+【会话劫持与凭证窃取】通过HTTP响应头注入，攻击者可构造恶意响应设置Cookie、重定向用户到钓鱼页面，或注入恶意JavaScript代码窃取用户会话令牌和登录凭证。
+【WAF/安全设备绕过】前端代理与后端forked-daapd/owntone-server对HTTP请求边界解析不一致，允许恶意请求绕过Web应用防火墙(WAF)的检测规则，直接到达后端服务器。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
         </is>
       </c>
     </row>
@@ -7111,6 +7457,14 @@
 5. 独立复现确认: replay_logical_vuln.sh — 71+ oracle违规验证</t>
         </is>
       </c>
+      <c r="K49" s="10" t="inlineStr">
+        <is>
+          <t>【HTTP缓存投毒】攻击者可利用forked-daapd/owntone-server的HTTP请求走私/响应分割漏洞，向前端缓存/代理服务器注入恶意HTTP响应，污染缓存内容。后续合法用户请求将收到被篡改的缓存内容，可能导致XSS、恶意重定向或恶意文件下载。
+【会话劫持与凭证窃取】通过HTTP响应头注入，攻击者可构造恶意响应设置Cookie、重定向用户到钓鱼页面，或注入恶意JavaScript代码窃取用户会话令牌和登录凭证。
+【WAF/安全设备绕过】前端代理与后端forked-daapd/owntone-server对HTTP请求边界解析不一致，允许恶意请求绕过Web应用防火墙(WAF)的检测规则，直接到达后端服务器。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="3" t="inlineStr">
@@ -7257,6 +7611,14 @@
 5. 独立复现确认: replay_logical_vuln.sh — 71+ oracle违规验证</t>
         </is>
       </c>
+      <c r="K50" s="10" t="inlineStr">
+        <is>
+          <t>【HTTP缓存投毒】攻击者可利用forked-daapd/owntone-server的HTTP请求走私/响应分割漏洞，向前端缓存/代理服务器注入恶意HTTP响应，污染缓存内容。后续合法用户请求将收到被篡改的缓存内容，可能导致XSS、恶意重定向或恶意文件下载。
+【会话劫持与凭证窃取】通过HTTP响应头注入，攻击者可构造恶意响应设置Cookie、重定向用户到钓鱼页面，或注入恶意JavaScript代码窃取用户会话令牌和登录凭证。
+【WAF/安全设备绕过】前端代理与后端forked-daapd/owntone-server对HTTP请求边界解析不一致，允许恶意请求绕过Web应用防火墙(WAF)的检测规则，直接到达后端服务器。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
@@ -7436,6 +7798,14 @@
 3. HTTP响应分割可导致缓存投毒、跨站脚本、页面劫持
 4. AFLNet协议Oracle检测到嵌入式HTTP响应模式
 5. 独立复现确认: replay_logical_vuln.sh — 8+ oracle违规验证</t>
+        </is>
+      </c>
+      <c r="K51" s="10" t="inlineStr">
+        <is>
+          <t>【HTTP缓存投毒】攻击者可利用forked-daapd/owntone-server的HTTP请求走私/响应分割漏洞，向前端缓存/代理服务器注入恶意HTTP响应，污染缓存内容。后续合法用户请求将收到被篡改的缓存内容，可能导致XSS、恶意重定向或恶意文件下载。
+【会话劫持与凭证窃取】通过HTTP响应头注入，攻击者可构造恶意响应设置Cookie、重定向用户到钓鱼页面，或注入恶意JavaScript代码窃取用户会话令牌和登录凭证。
+【WAF/安全设备绕过】前端代理与后端forked-daapd/owntone-server对HTTP请求边界解析不一致，允许恶意请求绕过Web应用防火墙(WAF)的检测规则，直接到达后端服务器。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
         </is>
       </c>
     </row>
@@ -7637,6 +8007,14 @@
 3. 攻击者可利用路径穿越访问任意文件系统资源
 4. AFLNet Oracle检测到路径穿越请求被服务器成功处理
 5. 独立复现确认: replay_logical_vuln.sh — 17+ oracle违规验证</t>
+        </is>
+      </c>
+      <c r="K52" s="10" t="inlineStr">
+        <is>
+          <t>【敏感文件读取】攻击者可利用forked-daapd/owntone-server的路径遍历漏洞读取服务器文件系统中的任意文件，包括/etc/passwd、/etc/shadow、SSH私钥、SSL证书私钥、应用配置文件（含数据库密码、API密钥）、日志文件（含会话令牌、用户IP）等高度敏感信息。
+【源代码泄露】若forked-daapd/owntone-server为Web/应用服务器，攻击者可读取应用源代码，从中发现更多安全漏洞（硬编码凭据、SQL注入点、反序列化入口等），形成漏洞利用链。
+【远程代码执行前置】路径遍历通常作为攻击链的第一阶段——攻击者读取配置文件获取凭据后，进一步通过SSH/数据库连接获取Shell，或利用读取到的密钥材料伪造签名/解密敏感通信。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
         </is>
       </c>
     </row>
@@ -7861,6 +8239,14 @@
 3. 攻击者可利用此绕过WAF/安全控制,窃取其他用户数据
 4. AFLNet协议Oracle在fuzzing中检测到CL desync违规
 5. 独立复现确认: replay_logical_vuln.sh — 71+ oracle违规验证</t>
+        </is>
+      </c>
+      <c r="K53" s="10" t="inlineStr">
+        <is>
+          <t>【HTTP缓存投毒】攻击者可利用forked-daapd/owntone-server的HTTP请求走私/响应分割漏洞，向前端缓存/代理服务器注入恶意HTTP响应，污染缓存内容。后续合法用户请求将收到被篡改的缓存内容，可能导致XSS、恶意重定向或恶意文件下载。
+【会话劫持与凭证窃取】通过HTTP响应头注入，攻击者可构造恶意响应设置Cookie、重定向用户到钓鱼页面，或注入恶意JavaScript代码窃取用户会话令牌和登录凭证。
+【WAF/安全设备绕过】前端代理与后端forked-daapd/owntone-server对HTTP请求边界解析不一致，允许恶意请求绕过Web应用防火墙(WAF)的检测规则，直接到达后端服务器。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
         </is>
       </c>
     </row>
@@ -8029,6 +8415,14 @@
 5. 独立复现确认: replay_logical_vuln.sh — 8+ oracle违规验证</t>
         </is>
       </c>
+      <c r="K54" s="10" t="inlineStr">
+        <is>
+          <t>【HTTP缓存投毒】攻击者可利用forked-daapd/owntone-server的HTTP请求走私/响应分割漏洞，向前端缓存/代理服务器注入恶意HTTP响应，污染缓存内容。后续合法用户请求将收到被篡改的缓存内容，可能导致XSS、恶意重定向或恶意文件下载。
+【会话劫持与凭证窃取】通过HTTP响应头注入，攻击者可构造恶意响应设置Cookie、重定向用户到钓鱼页面，或注入恶意JavaScript代码窃取用户会话令牌和登录凭证。
+【WAF/安全设备绕过】前端代理与后端forked-daapd/owntone-server对HTTP请求边界解析不一致，允许恶意请求绕过Web应用防火墙(WAF)的检测规则，直接到达后端服务器。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
@@ -8229,6 +8623,14 @@
 5. 独立复现确认: replay_logical_vuln.sh — 8+ oracle违规验证</t>
         </is>
       </c>
+      <c r="K55" s="10" t="inlineStr">
+        <is>
+          <t>【HTTP缓存投毒】攻击者可利用forked-daapd/owntone-server的HTTP请求走私/响应分割漏洞，向前端缓存/代理服务器注入恶意HTTP响应，污染缓存内容。后续合法用户请求将收到被篡改的缓存内容，可能导致XSS、恶意重定向或恶意文件下载。
+【会话劫持与凭证窃取】通过HTTP响应头注入，攻击者可构造恶意响应设置Cookie、重定向用户到钓鱼页面，或注入恶意JavaScript代码窃取用户会话令牌和登录凭证。
+【WAF/安全设备绕过】前端代理与后端forked-daapd/owntone-server对HTTP请求边界解析不一致，允许恶意请求绕过Web应用防火墙(WAF)的检测规则，直接到达后端服务器。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="3" t="inlineStr">
@@ -8441,6 +8843,14 @@
 5. 独立复现确认: replay_logical_vuln.sh — 71+ oracle违规验证</t>
         </is>
       </c>
+      <c r="K56" s="10" t="inlineStr">
+        <is>
+          <t>【HTTP缓存投毒】攻击者可利用forked-daapd/owntone-server的HTTP请求走私/响应分割漏洞，向前端缓存/代理服务器注入恶意HTTP响应，污染缓存内容。后续合法用户请求将收到被篡改的缓存内容，可能导致XSS、恶意重定向或恶意文件下载。
+【会话劫持与凭证窃取】通过HTTP响应头注入，攻击者可构造恶意响应设置Cookie、重定向用户到钓鱼页面，或注入恶意JavaScript代码窃取用户会话令牌和登录凭证。
+【WAF/安全设备绕过】前端代理与后端forked-daapd/owntone-server对HTTP请求边界解析不一致，允许恶意请求绕过Web应用防火墙(WAF)的检测规则，直接到达后端服务器。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="3" t="inlineStr">
@@ -8593,6 +9003,14 @@
 3. HTTP响应分割可导致缓存投毒、跨站脚本、页面劫持
 4. AFLNet协议Oracle检测到嵌入式HTTP响应模式
 5. 独立复现确认: replay_logical_vuln.sh — 8+ oracle违规验证</t>
+        </is>
+      </c>
+      <c r="K57" s="10" t="inlineStr">
+        <is>
+          <t>【HTTP缓存投毒】攻击者可利用forked-daapd/owntone-server的HTTP请求走私/响应分割漏洞，向前端缓存/代理服务器注入恶意HTTP响应，污染缓存内容。后续合法用户请求将收到被篡改的缓存内容，可能导致XSS、恶意重定向或恶意文件下载。
+【会话劫持与凭证窃取】通过HTTP响应头注入，攻击者可构造恶意响应设置Cookie、重定向用户到钓鱼页面，或注入恶意JavaScript代码窃取用户会话令牌和登录凭证。
+【WAF/安全设备绕过】前端代理与后端forked-daapd/owntone-server对HTTP请求边界解析不一致，允许恶意请求绕过Web应用防火墙(WAF)的检测规则，直接到达后端服务器。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
         </is>
       </c>
     </row>
@@ -8756,6 +9174,14 @@
 5. 独立复现确认: replay_logical_vuln.sh — 71+ oracle违规验证</t>
         </is>
       </c>
+      <c r="K58" s="10" t="inlineStr">
+        <is>
+          <t>【HTTP缓存投毒】攻击者可利用forked-daapd/owntone-server的HTTP请求走私/响应分割漏洞，向前端缓存/代理服务器注入恶意HTTP响应，污染缓存内容。后续合法用户请求将收到被篡改的缓存内容，可能导致XSS、恶意重定向或恶意文件下载。
+【会话劫持与凭证窃取】通过HTTP响应头注入，攻击者可构造恶意响应设置Cookie、重定向用户到钓鱼页面，或注入恶意JavaScript代码窃取用户会话令牌和登录凭证。
+【WAF/安全设备绕过】前端代理与后端forked-daapd/owntone-server对HTTP请求边界解析不一致，允许恶意请求绕过Web应用防火墙(WAF)的检测规则，直接到达后端服务器。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
@@ -8977,6 +9403,14 @@
 5. 独立复现确认: replay_logical_vuln.sh — 8+ oracle违规验证</t>
         </is>
       </c>
+      <c r="K59" s="10" t="inlineStr">
+        <is>
+          <t>【HTTP缓存投毒】攻击者可利用forked-daapd/owntone-server的HTTP请求走私/响应分割漏洞，向前端缓存/代理服务器注入恶意HTTP响应，污染缓存内容。后续合法用户请求将收到被篡改的缓存内容，可能导致XSS、恶意重定向或恶意文件下载。
+【会话劫持与凭证窃取】通过HTTP响应头注入，攻击者可构造恶意响应设置Cookie、重定向用户到钓鱼页面，或注入恶意JavaScript代码窃取用户会话令牌和登录凭证。
+【WAF/安全设备绕过】前端代理与后端forked-daapd/owntone-server对HTTP请求边界解析不一致，允许恶意请求绕过Web应用防火墙(WAF)的检测规则，直接到达后端服务器。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="3" t="inlineStr">
@@ -9190,6 +9624,14 @@
 5. 独立复现确认: replay_logical_vuln.sh — 71+ oracle违规验证</t>
         </is>
       </c>
+      <c r="K60" s="10" t="inlineStr">
+        <is>
+          <t>【HTTP缓存投毒】攻击者可利用forked-daapd/owntone-server的HTTP请求走私/响应分割漏洞，向前端缓存/代理服务器注入恶意HTTP响应，污染缓存内容。后续合法用户请求将收到被篡改的缓存内容，可能导致XSS、恶意重定向或恶意文件下载。
+【会话劫持与凭证窃取】通过HTTP响应头注入，攻击者可构造恶意响应设置Cookie、重定向用户到钓鱼页面，或注入恶意JavaScript代码窃取用户会话令牌和登录凭证。
+【WAF/安全设备绕过】前端代理与后端forked-daapd/owntone-server对HTTP请求边界解析不一致，允许恶意请求绕过Web应用防火墙(WAF)的检测规则，直接到达后端服务器。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="3" t="inlineStr">
@@ -9400,6 +9842,14 @@
 5. 独立复现确认: replay_logical_vuln.sh — 71+ oracle违规验证</t>
         </is>
       </c>
+      <c r="K61" s="10" t="inlineStr">
+        <is>
+          <t>【HTTP缓存投毒】攻击者可利用forked-daapd/owntone-server的HTTP请求走私/响应分割漏洞，向前端缓存/代理服务器注入恶意HTTP响应，污染缓存内容。后续合法用户请求将收到被篡改的缓存内容，可能导致XSS、恶意重定向或恶意文件下载。
+【会话劫持与凭证窃取】通过HTTP响应头注入，攻击者可构造恶意响应设置Cookie、重定向用户到钓鱼页面，或注入恶意JavaScript代码窃取用户会话令牌和登录凭证。
+【WAF/安全设备绕过】前端代理与后端forked-daapd/owntone-server对HTTP请求边界解析不一致，允许恶意请求绕过Web应用防火墙(WAF)的检测规则，直接到达后端服务器。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="3" t="inlineStr">
@@ -9660,6 +10110,14 @@
 5. 独立复现确认: replay_logical_vuln.sh — 8+ oracle违规验证</t>
         </is>
       </c>
+      <c r="K62" s="10" t="inlineStr">
+        <is>
+          <t>【HTTP缓存投毒】攻击者可利用forked-daapd/owntone-server的HTTP请求走私/响应分割漏洞，向前端缓存/代理服务器注入恶意HTTP响应，污染缓存内容。后续合法用户请求将收到被篡改的缓存内容，可能导致XSS、恶意重定向或恶意文件下载。
+【会话劫持与凭证窃取】通过HTTP响应头注入，攻击者可构造恶意响应设置Cookie、重定向用户到钓鱼页面，或注入恶意JavaScript代码窃取用户会话令牌和登录凭证。
+【WAF/安全设备绕过】前端代理与后端forked-daapd/owntone-server对HTTP请求边界解析不一致，允许恶意请求绕过Web应用防火墙(WAF)的检测规则，直接到达后端服务器。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="3" t="inlineStr">
@@ -9911,6 +10369,14 @@
 3. 攻击者可利用此绕过WAF/安全控制,窃取其他用户数据
 4. AFLNet协议Oracle在fuzzing中检测到CL desync违规
 5. 独立复现确认: replay_logical_vuln.sh — 71+ oracle违规验证</t>
+        </is>
+      </c>
+      <c r="K63" s="10" t="inlineStr">
+        <is>
+          <t>【HTTP缓存投毒】攻击者可利用forked-daapd/owntone-server的HTTP请求走私/响应分割漏洞，向前端缓存/代理服务器注入恶意HTTP响应，污染缓存内容。后续合法用户请求将收到被篡改的缓存内容，可能导致XSS、恶意重定向或恶意文件下载。
+【会话劫持与凭证窃取】通过HTTP响应头注入，攻击者可构造恶意响应设置Cookie、重定向用户到钓鱼页面，或注入恶意JavaScript代码窃取用户会话令牌和登录凭证。
+【WAF/安全设备绕过】前端代理与后端forked-daapd/owntone-server对HTTP请求边界解析不一致，允许恶意请求绕过Web应用防火墙(WAF)的检测规则，直接到达后端服务器。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
         </is>
       </c>
     </row>
@@ -10109,6 +10575,14 @@
 3. 攻击者可利用此绕过WAF/安全控制,窃取其他用户数据
 4. AFLNet协议Oracle在fuzzing中检测到CL desync违规
 5. 独立复现确认: replay_logical_vuln.sh — 71+ oracle违规验证</t>
+        </is>
+      </c>
+      <c r="K64" s="10" t="inlineStr">
+        <is>
+          <t>【HTTP缓存投毒】攻击者可利用forked-daapd/owntone-server的HTTP请求走私/响应分割漏洞，向前端缓存/代理服务器注入恶意HTTP响应，污染缓存内容。后续合法用户请求将收到被篡改的缓存内容，可能导致XSS、恶意重定向或恶意文件下载。
+【会话劫持与凭证窃取】通过HTTP响应头注入，攻击者可构造恶意响应设置Cookie、重定向用户到钓鱼页面，或注入恶意JavaScript代码窃取用户会话令牌和登录凭证。
+【WAF/安全设备绕过】前端代理与后端forked-daapd/owntone-server对HTTP请求边界解析不一致，允许恶意请求绕过Web应用防火墙(WAF)的检测规则，直接到达后端服务器。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
         </is>
       </c>
     </row>
@@ -10285,6 +10759,14 @@
 5. 独立复现确认: replay_logical_vuln.sh — 8+ oracle违规验证</t>
         </is>
       </c>
+      <c r="K65" s="10" t="inlineStr">
+        <is>
+          <t>【HTTP缓存投毒】攻击者可利用forked-daapd/owntone-server的HTTP请求走私/响应分割漏洞，向前端缓存/代理服务器注入恶意HTTP响应，污染缓存内容。后续合法用户请求将收到被篡改的缓存内容，可能导致XSS、恶意重定向或恶意文件下载。
+【会话劫持与凭证窃取】通过HTTP响应头注入，攻击者可构造恶意响应设置Cookie、重定向用户到钓鱼页面，或注入恶意JavaScript代码窃取用户会话令牌和登录凭证。
+【WAF/安全设备绕过】前端代理与后端forked-daapd/owntone-server对HTTP请求边界解析不一致，允许恶意请求绕过Web应用防火墙(WAF)的检测规则，直接到达后端服务器。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="3" t="inlineStr">
@@ -10529,6 +11011,14 @@
 5. 独立复现确认: replay_logical_vuln.sh — 71+ oracle违规验证</t>
         </is>
       </c>
+      <c r="K66" s="10" t="inlineStr">
+        <is>
+          <t>【HTTP缓存投毒】攻击者可利用forked-daapd/owntone-server的HTTP请求走私/响应分割漏洞，向前端缓存/代理服务器注入恶意HTTP响应，污染缓存内容。后续合法用户请求将收到被篡改的缓存内容，可能导致XSS、恶意重定向或恶意文件下载。
+【会话劫持与凭证窃取】通过HTTP响应头注入，攻击者可构造恶意响应设置Cookie、重定向用户到钓鱼页面，或注入恶意JavaScript代码窃取用户会话令牌和登录凭证。
+【WAF/安全设备绕过】前端代理与后端forked-daapd/owntone-server对HTTP请求边界解析不一致，允许恶意请求绕过Web应用防火墙(WAF)的检测规则，直接到达后端服务器。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="3" t="inlineStr">
@@ -10782,6 +11272,14 @@
 3. HTTP响应分割可导致缓存投毒、跨站脚本、页面劫持
 4. AFLNet协议Oracle检测到嵌入式HTTP响应模式
 5. 独立复现确认: replay_logical_vuln.sh — 8+ oracle违规验证</t>
+        </is>
+      </c>
+      <c r="K67" s="10" t="inlineStr">
+        <is>
+          <t>【HTTP缓存投毒】攻击者可利用forked-daapd/owntone-server的HTTP请求走私/响应分割漏洞，向前端缓存/代理服务器注入恶意HTTP响应，污染缓存内容。后续合法用户请求将收到被篡改的缓存内容，可能导致XSS、恶意重定向或恶意文件下载。
+【会话劫持与凭证窃取】通过HTTP响应头注入，攻击者可构造恶意响应设置Cookie、重定向用户到钓鱼页面，或注入恶意JavaScript代码窃取用户会话令牌和登录凭证。
+【WAF/安全设备绕过】前端代理与后端forked-daapd/owntone-server对HTTP请求边界解析不一致，允许恶意请求绕过Web应用防火墙(WAF)的检测规则，直接到达后端服务器。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
         </is>
       </c>
     </row>
@@ -10958,6 +11456,14 @@
 5. 独立复现确认: replay_logical_vuln.sh — 71+ oracle违规验证</t>
         </is>
       </c>
+      <c r="K68" s="10" t="inlineStr">
+        <is>
+          <t>【HTTP缓存投毒】攻击者可利用forked-daapd/owntone-server的HTTP请求走私/响应分割漏洞，向前端缓存/代理服务器注入恶意HTTP响应，污染缓存内容。后续合法用户请求将收到被篡改的缓存内容，可能导致XSS、恶意重定向或恶意文件下载。
+【会话劫持与凭证窃取】通过HTTP响应头注入，攻击者可构造恶意响应设置Cookie、重定向用户到钓鱼页面，或注入恶意JavaScript代码窃取用户会话令牌和登录凭证。
+【WAF/安全设备绕过】前端代理与后端forked-daapd/owntone-server对HTTP请求边界解析不一致，允许恶意请求绕过Web应用防火墙(WAF)的检测规则，直接到达后端服务器。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="3" t="inlineStr">
@@ -11071,6 +11577,14 @@
 3. 攻击者可利用此绕过WAF/安全控制,窃取其他用户数据
 4. AFLNet协议Oracle在fuzzing中检测到CL desync违规
 5. 独立复现确认: replay_logical_vuln.sh — 71+ oracle违规验证</t>
+        </is>
+      </c>
+      <c r="K69" s="10" t="inlineStr">
+        <is>
+          <t>【HTTP缓存投毒】攻击者可利用forked-daapd/owntone-server的HTTP请求走私/响应分割漏洞，向前端缓存/代理服务器注入恶意HTTP响应，污染缓存内容。后续合法用户请求将收到被篡改的缓存内容，可能导致XSS、恶意重定向或恶意文件下载。
+【会话劫持与凭证窃取】通过HTTP响应头注入，攻击者可构造恶意响应设置Cookie、重定向用户到钓鱼页面，或注入恶意JavaScript代码窃取用户会话令牌和登录凭证。
+【WAF/安全设备绕过】前端代理与后端forked-daapd/owntone-server对HTTP请求边界解析不一致，允许恶意请求绕过Web应用防火墙(WAF)的检测规则，直接到达后端服务器。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
         </is>
       </c>
     </row>
@@ -11222,6 +11736,14 @@
 3. HTTP响应分割可导致缓存投毒、跨站脚本、页面劫持
 4. AFLNet协议Oracle检测到嵌入式HTTP响应模式
 5. 独立复现确认: replay_logical_vuln.sh — 8+ oracle违规验证</t>
+        </is>
+      </c>
+      <c r="K70" s="10" t="inlineStr">
+        <is>
+          <t>【HTTP缓存投毒】攻击者可利用forked-daapd/owntone-server的HTTP请求走私/响应分割漏洞，向前端缓存/代理服务器注入恶意HTTP响应，污染缓存内容。后续合法用户请求将收到被篡改的缓存内容，可能导致XSS、恶意重定向或恶意文件下载。
+【会话劫持与凭证窃取】通过HTTP响应头注入，攻击者可构造恶意响应设置Cookie、重定向用户到钓鱼页面，或注入恶意JavaScript代码窃取用户会话令牌和登录凭证。
+【WAF/安全设备绕过】前端代理与后端forked-daapd/owntone-server对HTTP请求边界解析不一致，允许恶意请求绕过Web应用防火墙(WAF)的检测规则，直接到达后端服务器。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
         </is>
       </c>
     </row>
@@ -11337,6 +11859,14 @@
 5. 独立复现确认: replay_logical_vuln.sh — 200 OK响应确认绕过</t>
         </is>
       </c>
+      <c r="K71" s="10" t="inlineStr">
+        <is>
+          <t>【未授权访问】攻击者可绕过forked-daapd/owntone-server的身份认证机制，无需提供有效凭据即可访问受保护的服务功能和数据。这相当于将forked-daapd/owntone-server的认证门控完全失效，任何能够网络连接到服务的攻击者均可获得已认证用户的权限。
+【数据泄露与篡改】认证绕过后，攻击者可读取、修改、删除forked-daapd/owntone-server管理的所有数据，包括敏感配置文件、用户数据、媒体内容等。若forked-daapd/owntone-server连接到其他后端系统，攻击面将进一步扩大。
+【权限提升跳板】认证绕过通常可作为进一步攻击的跳板——攻击者获取立足点后可利用其他漏洞（如路径遍历、命令注入）扩大控制范围。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="3" t="inlineStr">
@@ -11476,6 +12006,14 @@
 3. 攻击者可利用此绕过WAF/安全控制,窃取其他用户数据
 4. AFLNet协议Oracle在fuzzing中检测到CL desync违规
 5. 独立复现确认: replay_logical_vuln.sh — 71+ oracle违规验证</t>
+        </is>
+      </c>
+      <c r="K72" s="10" t="inlineStr">
+        <is>
+          <t>【HTTP缓存投毒】攻击者可利用forked-daapd/owntone-server的HTTP请求走私/响应分割漏洞，向前端缓存/代理服务器注入恶意HTTP响应，污染缓存内容。后续合法用户请求将收到被篡改的缓存内容，可能导致XSS、恶意重定向或恶意文件下载。
+【会话劫持与凭证窃取】通过HTTP响应头注入，攻击者可构造恶意响应设置Cookie、重定向用户到钓鱼页面，或注入恶意JavaScript代码窃取用户会话令牌和登录凭证。
+【WAF/安全设备绕过】前端代理与后端forked-daapd/owntone-server对HTTP请求边界解析不一致，允许恶意请求绕过Web应用防火墙(WAF)的检测规则，直接到达后端服务器。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
         </is>
       </c>
     </row>
@@ -11581,6 +12119,14 @@
 3. HTTP响应分割可导致缓存投毒、跨站脚本、页面劫持
 4. AFLNet协议Oracle检测到嵌入式HTTP响应模式
 5. 独立复现确认: replay_logical_vuln.sh — 8+ oracle违规验证</t>
+        </is>
+      </c>
+      <c r="K73" s="10" t="inlineStr">
+        <is>
+          <t>【HTTP缓存投毒】攻击者可利用forked-daapd/owntone-server的HTTP请求走私/响应分割漏洞，向前端缓存/代理服务器注入恶意HTTP响应，污染缓存内容。后续合法用户请求将收到被篡改的缓存内容，可能导致XSS、恶意重定向或恶意文件下载。
+【会话劫持与凭证窃取】通过HTTP响应头注入，攻击者可构造恶意响应设置Cookie、重定向用户到钓鱼页面，或注入恶意JavaScript代码窃取用户会话令牌和登录凭证。
+【WAF/安全设备绕过】前端代理与后端forked-daapd/owntone-server对HTTP请求边界解析不一致，允许恶意请求绕过Web应用防火墙(WAF)的检测规则，直接到达后端服务器。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
         </is>
       </c>
     </row>
@@ -11690,6 +12236,14 @@
 5. 独立复现确认: replay_logical_vuln.sh — 8+ oracle违规验证</t>
         </is>
       </c>
+      <c r="K74" s="10" t="inlineStr">
+        <is>
+          <t>【HTTP缓存投毒】攻击者可利用forked-daapd/owntone-server的HTTP请求走私/响应分割漏洞，向前端缓存/代理服务器注入恶意HTTP响应，污染缓存内容。后续合法用户请求将收到被篡改的缓存内容，可能导致XSS、恶意重定向或恶意文件下载。
+【会话劫持与凭证窃取】通过HTTP响应头注入，攻击者可构造恶意响应设置Cookie、重定向用户到钓鱼页面，或注入恶意JavaScript代码窃取用户会话令牌和登录凭证。
+【WAF/安全设备绕过】前端代理与后端forked-daapd/owntone-server对HTTP请求边界解析不一致，允许恶意请求绕过Web应用防火墙(WAF)的检测规则，直接到达后端服务器。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="3" t="inlineStr">
@@ -11825,6 +12379,14 @@
 3. 攻击者可利用此绕过WAF/安全控制,窃取其他用户数据
 4. AFLNet协议Oracle在fuzzing中检测到CL desync违规
 5. 独立复现确认: replay_logical_vuln.sh — 71+ oracle违规验证</t>
+        </is>
+      </c>
+      <c r="K75" s="10" t="inlineStr">
+        <is>
+          <t>【HTTP缓存投毒】攻击者可利用forked-daapd/owntone-server的HTTP请求走私/响应分割漏洞，向前端缓存/代理服务器注入恶意HTTP响应，污染缓存内容。后续合法用户请求将收到被篡改的缓存内容，可能导致XSS、恶意重定向或恶意文件下载。
+【会话劫持与凭证窃取】通过HTTP响应头注入，攻击者可构造恶意响应设置Cookie、重定向用户到钓鱼页面，或注入恶意JavaScript代码窃取用户会话令牌和登录凭证。
+【WAF/安全设备绕过】前端代理与后端forked-daapd/owntone-server对HTTP请求边界解析不一致，允许恶意请求绕过Web应用防火墙(WAF)的检测规则，直接到达后端服务器。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
         </is>
       </c>
     </row>
@@ -11989,6 +12551,14 @@
 5. 独立复现确认: replay_logical_vuln.sh — 8+ oracle违规验证</t>
         </is>
       </c>
+      <c r="K76" s="10" t="inlineStr">
+        <is>
+          <t>【HTTP缓存投毒】攻击者可利用forked-daapd/owntone-server的HTTP请求走私/响应分割漏洞，向前端缓存/代理服务器注入恶意HTTP响应，污染缓存内容。后续合法用户请求将收到被篡改的缓存内容，可能导致XSS、恶意重定向或恶意文件下载。
+【会话劫持与凭证窃取】通过HTTP响应头注入，攻击者可构造恶意响应设置Cookie、重定向用户到钓鱼页面，或注入恶意JavaScript代码窃取用户会话令牌和登录凭证。
+【WAF/安全设备绕过】前端代理与后端forked-daapd/owntone-server对HTTP请求边界解析不一致，允许恶意请求绕过Web应用防火墙(WAF)的检测规则，直接到达后端服务器。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="3" t="inlineStr">
@@ -12144,6 +12714,14 @@
 5. 独立复现确认: replay_logical_vuln.sh — 71+ oracle违规验证</t>
         </is>
       </c>
+      <c r="K77" s="10" t="inlineStr">
+        <is>
+          <t>【HTTP缓存投毒】攻击者可利用forked-daapd/owntone-server的HTTP请求走私/响应分割漏洞，向前端缓存/代理服务器注入恶意HTTP响应，污染缓存内容。后续合法用户请求将收到被篡改的缓存内容，可能导致XSS、恶意重定向或恶意文件下载。
+【会话劫持与凭证窃取】通过HTTP响应头注入，攻击者可构造恶意响应设置Cookie、重定向用户到钓鱼页面，或注入恶意JavaScript代码窃取用户会话令牌和登录凭证。
+【WAF/安全设备绕过】前端代理与后端forked-daapd/owntone-server对HTTP请求边界解析不一致，允许恶意请求绕过Web应用防火墙(WAF)的检测规则，直接到达后端服务器。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="3" t="inlineStr">
@@ -12247,6 +12825,14 @@
 3. 攻击者可利用此绕过WAF/安全控制,窃取其他用户数据
 4. AFLNet协议Oracle在fuzzing中检测到CL desync违规
 5. 独立复现确认: replay_logical_vuln.sh — 71+ oracle违规验证</t>
+        </is>
+      </c>
+      <c r="K78" s="10" t="inlineStr">
+        <is>
+          <t>【HTTP缓存投毒】攻击者可利用forked-daapd/owntone-server的HTTP请求走私/响应分割漏洞，向前端缓存/代理服务器注入恶意HTTP响应，污染缓存内容。后续合法用户请求将收到被篡改的缓存内容，可能导致XSS、恶意重定向或恶意文件下载。
+【会话劫持与凭证窃取】通过HTTP响应头注入，攻击者可构造恶意响应设置Cookie、重定向用户到钓鱼页面，或注入恶意JavaScript代码窃取用户会话令牌和登录凭证。
+【WAF/安全设备绕过】前端代理与后端forked-daapd/owntone-server对HTTP请求边界解析不一致，允许恶意请求绕过Web应用防火墙(WAF)的检测规则，直接到达后端服务器。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
         </is>
       </c>
     </row>
@@ -12459,6 +13045,14 @@
 5. 独立复现确认: replay_logical_vuln.sh — 8+ oracle违规验证</t>
         </is>
       </c>
+      <c r="K79" s="10" t="inlineStr">
+        <is>
+          <t>【HTTP缓存投毒】攻击者可利用forked-daapd/owntone-server的HTTP请求走私/响应分割漏洞，向前端缓存/代理服务器注入恶意HTTP响应，污染缓存内容。后续合法用户请求将收到被篡改的缓存内容，可能导致XSS、恶意重定向或恶意文件下载。
+【会话劫持与凭证窃取】通过HTTP响应头注入，攻击者可构造恶意响应设置Cookie、重定向用户到钓鱼页面，或注入恶意JavaScript代码窃取用户会话令牌和登录凭证。
+【WAF/安全设备绕过】前端代理与后端forked-daapd/owntone-server对HTTP请求边界解析不一致，允许恶意请求绕过Web应用防火墙(WAF)的检测规则，直接到达后端服务器。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="3" t="inlineStr">
@@ -12569,6 +13163,14 @@
 5. 独立复现确认: replay_logical_vuln.sh — 200 OK响应确认绕过</t>
         </is>
       </c>
+      <c r="K80" s="10" t="inlineStr">
+        <is>
+          <t>【未授权访问】攻击者可绕过forked-daapd/owntone-server的身份认证机制，无需提供有效凭据即可访问受保护的服务功能和数据。这相当于将forked-daapd/owntone-server的认证门控完全失效，任何能够网络连接到服务的攻击者均可获得已认证用户的权限。
+【数据泄露与篡改】认证绕过后，攻击者可读取、修改、删除forked-daapd/owntone-server管理的所有数据，包括敏感配置文件、用户数据、媒体内容等。若forked-daapd/owntone-server连接到其他后端系统，攻击面将进一步扩大。
+【权限提升跳板】认证绕过通常可作为进一步攻击的跳板——攻击者获取立足点后可利用其他漏洞（如路径遍历、命令注入）扩大控制范围。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="3" t="inlineStr">
@@ -12708,6 +13310,14 @@
 5. 独立复现确认: replay_logical_vuln.sh — 71+ oracle违规验证</t>
         </is>
       </c>
+      <c r="K81" s="10" t="inlineStr">
+        <is>
+          <t>【HTTP缓存投毒】攻击者可利用forked-daapd/owntone-server的HTTP请求走私/响应分割漏洞，向前端缓存/代理服务器注入恶意HTTP响应，污染缓存内容。后续合法用户请求将收到被篡改的缓存内容，可能导致XSS、恶意重定向或恶意文件下载。
+【会话劫持与凭证窃取】通过HTTP响应头注入，攻击者可构造恶意响应设置Cookie、重定向用户到钓鱼页面，或注入恶意JavaScript代码窃取用户会话令牌和登录凭证。
+【WAF/安全设备绕过】前端代理与后端forked-daapd/owntone-server对HTTP请求边界解析不一致，允许恶意请求绕过Web应用防火墙(WAF)的检测规则，直接到达后端服务器。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="3" t="inlineStr">
@@ -12881,6 +13491,14 @@
 3. HTTP响应分割可导致缓存投毒、跨站脚本、页面劫持
 4. AFLNet协议Oracle检测到嵌入式HTTP响应模式
 5. 独立复现确认: replay_logical_vuln.sh — 8+ oracle违规验证</t>
+        </is>
+      </c>
+      <c r="K82" s="10" t="inlineStr">
+        <is>
+          <t>【HTTP缓存投毒】攻击者可利用forked-daapd/owntone-server的HTTP请求走私/响应分割漏洞，向前端缓存/代理服务器注入恶意HTTP响应，污染缓存内容。后续合法用户请求将收到被篡改的缓存内容，可能导致XSS、恶意重定向或恶意文件下载。
+【会话劫持与凭证窃取】通过HTTP响应头注入，攻击者可构造恶意响应设置Cookie、重定向用户到钓鱼页面，或注入恶意JavaScript代码窃取用户会话令牌和登录凭证。
+【WAF/安全设备绕过】前端代理与后端forked-daapd/owntone-server对HTTP请求边界解析不一致，允许恶意请求绕过Web应用防火墙(WAF)的检测规则，直接到达后端服务器。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
         </is>
       </c>
     </row>
@@ -13071,6 +13689,14 @@
 5. 独立复现确认: replay_logical_vuln.sh — 71+ oracle违规验证</t>
         </is>
       </c>
+      <c r="K83" s="10" t="inlineStr">
+        <is>
+          <t>【HTTP缓存投毒】攻击者可利用forked-daapd/owntone-server的HTTP请求走私/响应分割漏洞，向前端缓存/代理服务器注入恶意HTTP响应，污染缓存内容。后续合法用户请求将收到被篡改的缓存内容，可能导致XSS、恶意重定向或恶意文件下载。
+【会话劫持与凭证窃取】通过HTTP响应头注入，攻击者可构造恶意响应设置Cookie、重定向用户到钓鱼页面，或注入恶意JavaScript代码窃取用户会话令牌和登录凭证。
+【WAF/安全设备绕过】前端代理与后端forked-daapd/owntone-server对HTTP请求边界解析不一致，允许恶意请求绕过Web应用防火墙(WAF)的检测规则，直接到达后端服务器。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="3" t="inlineStr">
@@ -13196,6 +13822,14 @@
 3. 攻击者可利用此绕过WAF/安全控制,窃取其他用户数据
 4. AFLNet协议Oracle在fuzzing中检测到CL desync违规
 5. 独立复现确认: replay_logical_vuln.sh — 71+ oracle违规验证</t>
+        </is>
+      </c>
+      <c r="K84" s="10" t="inlineStr">
+        <is>
+          <t>【HTTP缓存投毒】攻击者可利用forked-daapd/owntone-server的HTTP请求走私/响应分割漏洞，向前端缓存/代理服务器注入恶意HTTP响应，污染缓存内容。后续合法用户请求将收到被篡改的缓存内容，可能导致XSS、恶意重定向或恶意文件下载。
+【会话劫持与凭证窃取】通过HTTP响应头注入，攻击者可构造恶意响应设置Cookie、重定向用户到钓鱼页面，或注入恶意JavaScript代码窃取用户会话令牌和登录凭证。
+【WAF/安全设备绕过】前端代理与后端forked-daapd/owntone-server对HTTP请求边界解析不一致，允许恶意请求绕过Web应用防火墙(WAF)的检测规则，直接到达后端服务器。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
         </is>
       </c>
     </row>
@@ -13404,6 +14038,14 @@
 5. 独立复现确认: replay_logical_vuln.sh — 8+ oracle违规验证</t>
         </is>
       </c>
+      <c r="K85" s="10" t="inlineStr">
+        <is>
+          <t>【HTTP缓存投毒】攻击者可利用forked-daapd/owntone-server的HTTP请求走私/响应分割漏洞，向前端缓存/代理服务器注入恶意HTTP响应，污染缓存内容。后续合法用户请求将收到被篡改的缓存内容，可能导致XSS、恶意重定向或恶意文件下载。
+【会话劫持与凭证窃取】通过HTTP响应头注入，攻击者可构造恶意响应设置Cookie、重定向用户到钓鱼页面，或注入恶意JavaScript代码窃取用户会话令牌和登录凭证。
+【WAF/安全设备绕过】前端代理与后端forked-daapd/owntone-server对HTTP请求边界解析不一致，允许恶意请求绕过Web应用防火墙(WAF)的检测规则，直接到达后端服务器。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="3" t="inlineStr">
@@ -13649,6 +14291,14 @@
 5. 独立复现确认: replay_logical_vuln.sh — 71+ oracle违规验证</t>
         </is>
       </c>
+      <c r="K86" s="10" t="inlineStr">
+        <is>
+          <t>【HTTP缓存投毒】攻击者可利用forked-daapd/owntone-server的HTTP请求走私/响应分割漏洞，向前端缓存/代理服务器注入恶意HTTP响应，污染缓存内容。后续合法用户请求将收到被篡改的缓存内容，可能导致XSS、恶意重定向或恶意文件下载。
+【会话劫持与凭证窃取】通过HTTP响应头注入，攻击者可构造恶意响应设置Cookie、重定向用户到钓鱼页面，或注入恶意JavaScript代码窃取用户会话令牌和登录凭证。
+【WAF/安全设备绕过】前端代理与后端forked-daapd/owntone-server对HTTP请求边界解析不一致，允许恶意请求绕过Web应用防火墙(WAF)的检测规则，直接到达后端服务器。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="3" t="inlineStr">
@@ -13866,6 +14516,14 @@
 3. 攻击者可利用此绕过WAF/安全控制,窃取其他用户数据
 4. AFLNet协议Oracle在fuzzing中检测到CL desync违规
 5. 独立复现确认: replay_logical_vuln.sh — 71+ oracle违规验证</t>
+        </is>
+      </c>
+      <c r="K87" s="10" t="inlineStr">
+        <is>
+          <t>【HTTP缓存投毒】攻击者可利用forked-daapd/owntone-server的HTTP请求走私/响应分割漏洞，向前端缓存/代理服务器注入恶意HTTP响应，污染缓存内容。后续合法用户请求将收到被篡改的缓存内容，可能导致XSS、恶意重定向或恶意文件下载。
+【会话劫持与凭证窃取】通过HTTP响应头注入，攻击者可构造恶意响应设置Cookie、重定向用户到钓鱼页面，或注入恶意JavaScript代码窃取用户会话令牌和登录凭证。
+【WAF/安全设备绕过】前端代理与后端forked-daapd/owntone-server对HTTP请求边界解析不一致，允许恶意请求绕过Web应用防火墙(WAF)的检测规则，直接到达后端服务器。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
         </is>
       </c>
     </row>
@@ -13990,6 +14648,14 @@
 5. 独立复现确认: replay_logical_vuln.sh — 8+ oracle违规验证</t>
         </is>
       </c>
+      <c r="K88" s="10" t="inlineStr">
+        <is>
+          <t>【HTTP缓存投毒】攻击者可利用forked-daapd/owntone-server的HTTP请求走私/响应分割漏洞，向前端缓存/代理服务器注入恶意HTTP响应，污染缓存内容。后续合法用户请求将收到被篡改的缓存内容，可能导致XSS、恶意重定向或恶意文件下载。
+【会话劫持与凭证窃取】通过HTTP响应头注入，攻击者可构造恶意响应设置Cookie、重定向用户到钓鱼页面，或注入恶意JavaScript代码窃取用户会话令牌和登录凭证。
+【WAF/安全设备绕过】前端代理与后端forked-daapd/owntone-server对HTTP请求边界解析不一致，允许恶意请求绕过Web应用防火墙(WAF)的检测规则，直接到达后端服务器。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="3" t="inlineStr">
@@ -14109,6 +14775,14 @@
 5. 独立复现确认: replay_logical_vuln.sh — 200 OK响应确认绕过</t>
         </is>
       </c>
+      <c r="K89" s="10" t="inlineStr">
+        <is>
+          <t>【未授权访问】攻击者可绕过forked-daapd/owntone-server的身份认证机制，无需提供有效凭据即可访问受保护的服务功能和数据。这相当于将forked-daapd/owntone-server的认证门控完全失效，任何能够网络连接到服务的攻击者均可获得已认证用户的权限。
+【数据泄露与篡改】认证绕过后，攻击者可读取、修改、删除forked-daapd/owntone-server管理的所有数据，包括敏感配置文件、用户数据、媒体内容等。若forked-daapd/owntone-server连接到其他后端系统，攻击面将进一步扩大。
+【权限提升跳板】认证绕过通常可作为进一步攻击的跳板——攻击者获取立足点后可利用其他漏洞（如路径遍历、命令注入）扩大控制范围。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="3" t="inlineStr">
@@ -14237,6 +14911,14 @@
 3. 攻击者可利用此绕过WAF/安全控制,窃取其他用户数据
 4. AFLNet协议Oracle在fuzzing中检测到CL desync违规
 5. 独立复现确认: replay_logical_vuln.sh — 71+ oracle违规验证</t>
+        </is>
+      </c>
+      <c r="K90" s="10" t="inlineStr">
+        <is>
+          <t>【HTTP缓存投毒】攻击者可利用forked-daapd/owntone-server的HTTP请求走私/响应分割漏洞，向前端缓存/代理服务器注入恶意HTTP响应，污染缓存内容。后续合法用户请求将收到被篡改的缓存内容，可能导致XSS、恶意重定向或恶意文件下载。
+【会话劫持与凭证窃取】通过HTTP响应头注入，攻击者可构造恶意响应设置Cookie、重定向用户到钓鱼页面，或注入恶意JavaScript代码窃取用户会话令牌和登录凭证。
+【WAF/安全设备绕过】前端代理与后端forked-daapd/owntone-server对HTTP请求边界解析不一致，允许恶意请求绕过Web应用防火墙(WAF)的检测规则，直接到达后端服务器。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
         </is>
       </c>
     </row>
@@ -14436,6 +15118,14 @@
 5. 独立复现确认: replay_logical_vuln.sh — 8+ oracle违规验证</t>
         </is>
       </c>
+      <c r="K91" s="10" t="inlineStr">
+        <is>
+          <t>【HTTP缓存投毒】攻击者可利用forked-daapd/owntone-server的HTTP请求走私/响应分割漏洞，向前端缓存/代理服务器注入恶意HTTP响应，污染缓存内容。后续合法用户请求将收到被篡改的缓存内容，可能导致XSS、恶意重定向或恶意文件下载。
+【会话劫持与凭证窃取】通过HTTP响应头注入，攻击者可构造恶意响应设置Cookie、重定向用户到钓鱼页面，或注入恶意JavaScript代码窃取用户会话令牌和登录凭证。
+【WAF/安全设备绕过】前端代理与后端forked-daapd/owntone-server对HTTP请求边界解析不一致，允许恶意请求绕过Web应用防火墙(WAF)的检测规则，直接到达后端服务器。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="3" t="inlineStr">
@@ -14542,6 +15232,14 @@
 3. 攻击者可利用此绕过WAF/安全控制,窃取其他用户数据
 4. AFLNet协议Oracle在fuzzing中检测到CL desync违规
 5. 独立复现确认: replay_logical_vuln.sh — 71+ oracle违规验证</t>
+        </is>
+      </c>
+      <c r="K92" s="10" t="inlineStr">
+        <is>
+          <t>【HTTP缓存投毒】攻击者可利用forked-daapd/owntone-server的HTTP请求走私/响应分割漏洞，向前端缓存/代理服务器注入恶意HTTP响应，污染缓存内容。后续合法用户请求将收到被篡改的缓存内容，可能导致XSS、恶意重定向或恶意文件下载。
+【会话劫持与凭证窃取】通过HTTP响应头注入，攻击者可构造恶意响应设置Cookie、重定向用户到钓鱼页面，或注入恶意JavaScript代码窃取用户会话令牌和登录凭证。
+【WAF/安全设备绕过】前端代理与后端forked-daapd/owntone-server对HTTP请求边界解析不一致，允许恶意请求绕过Web应用防火墙(WAF)的检测规则，直接到达后端服务器。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
         </is>
       </c>
     </row>
@@ -14667,6 +15365,14 @@
 5. 独立复现确认: replay_logical_vuln.sh — 8+ oracle违规验证</t>
         </is>
       </c>
+      <c r="K93" s="10" t="inlineStr">
+        <is>
+          <t>【HTTP缓存投毒】攻击者可利用forked-daapd/owntone-server的HTTP请求走私/响应分割漏洞，向前端缓存/代理服务器注入恶意HTTP响应，污染缓存内容。后续合法用户请求将收到被篡改的缓存内容，可能导致XSS、恶意重定向或恶意文件下载。
+【会话劫持与凭证窃取】通过HTTP响应头注入，攻击者可构造恶意响应设置Cookie、重定向用户到钓鱼页面，或注入恶意JavaScript代码窃取用户会话令牌和登录凭证。
+【WAF/安全设备绕过】前端代理与后端forked-daapd/owntone-server对HTTP请求边界解析不一致，允许恶意请求绕过Web应用防火墙(WAF)的检测规则，直接到达后端服务器。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="4" t="inlineStr">
@@ -14747,6 +15453,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K94" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="4" t="inlineStr">
@@ -14827,6 +15539,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K95" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="4" t="inlineStr">
@@ -14907,6 +15625,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K96" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="4" t="inlineStr">
@@ -14987,6 +15711,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K97" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="4" t="inlineStr">
@@ -15067,6 +15797,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K98" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="4" t="inlineStr">
@@ -15147,6 +15883,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K99" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="4" t="inlineStr">
@@ -15227,6 +15969,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K100" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="4" t="inlineStr">
@@ -15307,6 +16055,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K101" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="4" t="inlineStr">
@@ -15387,6 +16141,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K102" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="4" t="inlineStr">
@@ -15467,6 +16227,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K103" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="4" t="inlineStr">
@@ -15547,6 +16313,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K104" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="4" t="inlineStr">
@@ -15627,6 +16399,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K105" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="4" t="inlineStr">
@@ -15707,6 +16485,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K106" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="4" t="inlineStr">
@@ -15787,6 +16571,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K107" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="4" t="inlineStr">
@@ -15867,6 +16657,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K108" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="4" t="inlineStr">
@@ -15947,6 +16743,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K109" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="4" t="inlineStr">
@@ -16027,6 +16829,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K110" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="4" t="inlineStr">
@@ -16107,6 +16915,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K111" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="4" t="inlineStr">
@@ -16187,6 +17001,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K112" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="4" t="inlineStr">
@@ -16267,6 +17087,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K113" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="4" t="inlineStr">
@@ -16347,6 +17173,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K114" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="4" t="inlineStr">
@@ -16427,6 +17259,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K115" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="4" t="inlineStr">
@@ -16507,6 +17345,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K116" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="4" t="inlineStr">
@@ -16587,6 +17431,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K117" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="4" t="inlineStr">
@@ -16667,6 +17517,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K118" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="4" t="inlineStr">
@@ -16747,6 +17603,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K119" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="4" t="inlineStr">
@@ -16827,6 +17689,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K120" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="4" t="inlineStr">
@@ -16907,6 +17775,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K121" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="4" t="inlineStr">
@@ -16987,6 +17861,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K122" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="4" t="inlineStr">
@@ -17067,6 +17947,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K123" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="4" t="inlineStr">
@@ -17147,6 +18033,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K124" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="4" t="inlineStr">
@@ -17227,6 +18119,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K125" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="4" t="inlineStr">
@@ -17307,6 +18205,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K126" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="4" t="inlineStr">
@@ -17387,6 +18291,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K127" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="4" t="inlineStr">
@@ -17467,6 +18377,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K128" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="4" t="inlineStr">
@@ -17547,6 +18463,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K129" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="4" t="inlineStr">
@@ -17627,6 +18549,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K130" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="4" t="inlineStr">
@@ -17707,6 +18635,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K131" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="4" t="inlineStr">
@@ -17787,6 +18721,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K132" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="4" t="inlineStr">
@@ -17867,6 +18807,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K133" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="4" t="inlineStr">
@@ -17947,6 +18893,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K134" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="4" t="inlineStr">
@@ -18027,6 +18979,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K135" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="4" t="inlineStr">
@@ -18107,6 +19065,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K136" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="4" t="inlineStr">
@@ -18187,6 +19151,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K137" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="4" t="inlineStr">
@@ -18267,6 +19237,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K138" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="4" t="inlineStr">
@@ -18347,6 +19323,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K139" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="4" t="inlineStr">
@@ -18427,6 +19409,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K140" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="4" t="inlineStr">
@@ -18507,6 +19495,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K141" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="4" t="inlineStr">
@@ -18587,6 +19581,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K142" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="4" t="inlineStr">
@@ -18667,6 +19667,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K143" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="4" t="inlineStr">
@@ -18747,6 +19753,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K144" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="4" t="inlineStr">
@@ -18827,6 +19839,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K145" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="4" t="inlineStr">
@@ -18907,6 +19925,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K146" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="4" t="inlineStr">
@@ -18987,6 +20011,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K147" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="4" t="inlineStr">
@@ -19067,6 +20097,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K148" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="4" t="inlineStr">
@@ -19147,6 +20183,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K149" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="4" t="inlineStr">
@@ -19227,6 +20269,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K150" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="4" t="inlineStr">
@@ -19307,6 +20355,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K151" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="4" t="inlineStr">
@@ -19387,6 +20441,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K152" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="4" t="inlineStr">
@@ -19467,6 +20527,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K153" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="4" t="inlineStr">
@@ -19547,6 +20613,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K154" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="4" t="inlineStr">
@@ -19627,6 +20699,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K155" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="4" t="inlineStr">
@@ -19707,6 +20785,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K156" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="4" t="inlineStr">
@@ -19787,6 +20871,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K157" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="4" t="inlineStr">
@@ -19867,6 +20957,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K158" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="4" t="inlineStr">
@@ -19947,6 +21043,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K159" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="4" t="inlineStr">
@@ -20027,6 +21129,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K160" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="4" t="inlineStr">
@@ -20107,6 +21215,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K161" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="4" t="inlineStr">
@@ -20187,6 +21301,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K162" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="4" t="inlineStr">
@@ -20267,6 +21387,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K163" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="4" t="inlineStr">
@@ -20347,6 +21473,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K164" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="4" t="inlineStr">
@@ -20427,6 +21559,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K165" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="166">
       <c r="A166" s="4" t="inlineStr">
@@ -20507,6 +21645,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K166" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="167">
       <c r="A167" s="4" t="inlineStr">
@@ -20587,6 +21731,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K167" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="168">
       <c r="A168" s="4" t="inlineStr">
@@ -20667,6 +21817,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K168" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" s="4" t="inlineStr">
@@ -20747,6 +21903,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K169" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="170">
       <c r="A170" s="4" t="inlineStr">
@@ -20827,6 +21989,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K170" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" s="4" t="inlineStr">
@@ -20907,6 +22075,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K171" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="172">
       <c r="A172" s="4" t="inlineStr">
@@ -20987,6 +22161,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K172" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="173">
       <c r="A173" s="4" t="inlineStr">
@@ -21067,6 +22247,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K173" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="174">
       <c r="A174" s="4" t="inlineStr">
@@ -21147,6 +22333,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K174" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="175">
       <c r="A175" s="4" t="inlineStr">
@@ -21227,6 +22419,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K175" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="176">
       <c r="A176" s="4" t="inlineStr">
@@ -21307,6 +22505,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K176" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="177">
       <c r="A177" s="4" t="inlineStr">
@@ -21387,6 +22591,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K177" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="178">
       <c r="A178" s="4" t="inlineStr">
@@ -21467,6 +22677,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K178" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="179">
       <c r="A179" s="4" t="inlineStr">
@@ -21547,6 +22763,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K179" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="180">
       <c r="A180" s="4" t="inlineStr">
@@ -21627,6 +22849,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K180" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="181">
       <c r="A181" s="4" t="inlineStr">
@@ -21707,6 +22935,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K181" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="182">
       <c r="A182" s="4" t="inlineStr">
@@ -21787,6 +23021,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K182" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="183">
       <c r="A183" s="4" t="inlineStr">
@@ -21867,6 +23107,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K183" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="184">
       <c r="A184" s="4" t="inlineStr">
@@ -21947,6 +23193,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K184" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="185">
       <c r="A185" s="4" t="inlineStr">
@@ -22027,6 +23279,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K185" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="186">
       <c r="A186" s="4" t="inlineStr">
@@ -22107,6 +23365,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K186" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="187">
       <c r="A187" s="4" t="inlineStr">
@@ -22187,6 +23451,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K187" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="188">
       <c r="A188" s="4" t="inlineStr">
@@ -22267,6 +23537,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K188" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="189">
       <c r="A189" s="4" t="inlineStr">
@@ -22347,6 +23623,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K189" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="190">
       <c r="A190" s="4" t="inlineStr">
@@ -22427,6 +23709,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K190" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="191">
       <c r="A191" s="4" t="inlineStr">
@@ -22507,6 +23795,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K191" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="192">
       <c r="A192" s="4" t="inlineStr">
@@ -22587,6 +23881,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K192" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="193">
       <c r="A193" s="4" t="inlineStr">
@@ -22667,6 +23967,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K193" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="194">
       <c r="A194" s="4" t="inlineStr">
@@ -22747,6 +24053,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K194" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="195">
       <c r="A195" s="4" t="inlineStr">
@@ -22827,6 +24139,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K195" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="196">
       <c r="A196" s="4" t="inlineStr">
@@ -22907,6 +24225,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K196" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="197">
       <c r="A197" s="4" t="inlineStr">
@@ -22987,6 +24311,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K197" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="198">
       <c r="A198" s="4" t="inlineStr">
@@ -23067,6 +24397,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K198" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="199">
       <c r="A199" s="4" t="inlineStr">
@@ -23147,6 +24483,12 @@
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
         </is>
       </c>
+      <c r="K199" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
+        </is>
+      </c>
     </row>
     <row r="200">
       <c r="A200" s="4" t="inlineStr">
@@ -23225,6 +24567,12 @@
 3. 远程攻击者可通过发送特定DAAP/HTTP请求序列导致服务器无法响应合法请求
 4. 10组独立实验每组均发现7-13个hang种子(100%覆盖率)
 5. 同类CVE(CVE-2025-63647/63648/57156, CVSS 7.5+)佐证owntone-server存在多个DoS弱点</t>
+        </is>
+      </c>
+      <c r="K200" s="10" t="inlineStr">
+        <is>
+          <t>【内存耗尽型拒绝服务】攻击者可向forked-daapd/owntone-server发送特制的超长协议字段或大量并发请求，导致服务器内存分配持续增长直至OOM(Out of Memory)。操作系统OOM Killer将强制终止forked-daapd/owntone-server进程，造成服务完全中断。在容器化部署环境中，可能触发Pod/容器重启，影响同节点其他服务。
+【漏洞可靠性高】AFLNet fuzzing框架已多次重放验证该漏洞的稳定性（标记为replayable），表明攻击者可在真实环境中稳定复现该漏洞，利用成功率较高。</t>
         </is>
       </c>
     </row>

</xml_diff>